<commit_message>
Update case import prototype
</commit_message>
<xml_diff>
--- a/problem_detail.xlsx
+++ b/problem_detail.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题明细" sheetId="1" r:id="Rfd7ca3301cb14b81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R6509f346d709423d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题明细" sheetId="1" r:id="Ra0f197927dd74a51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R9f4aab17190644ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -127,9 +127,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -142,12 +142,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -241,15 +287,11 @@
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="8" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="8" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="12" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="8" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="8" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="40" customHeight="1">
@@ -269,40 +311,28 @@
         <x:v>客户姓名</x:v>
       </x:c>
       <x:c r="F1" s="8" t="str">
-        <x:v>处理环节</x:v>
+        <x:v>导入结果</x:v>
       </x:c>
       <x:c r="G1" s="8" t="str">
-        <x:v>导入结果</x:v>
+        <x:v>问题类型</x:v>
       </x:c>
       <x:c r="H1" s="8" t="str">
-        <x:v>问题类型</x:v>
+        <x:v>字段路径</x:v>
       </x:c>
       <x:c r="I1" s="8" t="str">
-        <x:v>字段路径</x:v>
+        <x:v>当前值</x:v>
       </x:c>
       <x:c r="J1" s="8" t="str">
-        <x:v>当前值</x:v>
+        <x:v>问题说明</x:v>
       </x:c>
       <x:c r="K1" s="8" t="str">
-        <x:v>问题说明</x:v>
+        <x:v>是否阻断导入</x:v>
       </x:c>
       <x:c r="L1" s="8" t="str">
-        <x:v>建议处理</x:v>
+        <x:v>材料项</x:v>
       </x:c>
       <x:c r="M1" s="8" t="str">
-        <x:v>是否阻断导入</x:v>
-      </x:c>
-      <x:c r="N1" s="8" t="str">
-        <x:v>材料项</x:v>
-      </x:c>
-      <x:c r="O1" s="8" t="str">
         <x:v>导入时间</x:v>
-      </x:c>
-      <x:c r="P1" s="8" t="str">
-        <x:v>处理状态</x:v>
-      </x:c>
-      <x:c r="Q1" s="8" t="str">
-        <x:v>备注</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -322,38 +352,26 @@
         <x:v>张三</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str">
-        <x:v>资产明细检查</x:v>
+        <x:v>重复待确认</x:v>
       </x:c>
       <x:c r="G2" s="9" t="str">
-        <x:v>阻断失败</x:v>
+        <x:v>重复待确认</x:v>
       </x:c>
       <x:c r="H2" s="9" t="str">
-        <x:v>账单期次重复</x:v>
+        <x:v>订单基础信息-订单编号</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>账单信息-期次</x:v>
+        <x:v>26012915050167612327</x:v>
       </x:c>
       <x:c r="J2" s="9" t="str">
-        <x:v>第3期重复</x:v>
+        <x:v>系统已存在同外部资产方、同订单编号案件，本次不新增案件、不自动覆盖字段和材料</x:v>
       </x:c>
       <x:c r="K2" s="9" t="str">
-        <x:v>同一订单第3期出现2次</x:v>
-      </x:c>
-      <x:c r="L2" s="9" t="str">
-        <x:v>修改模板后重新上传</x:v>
-      </x:c>
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="L2" s="9" t="str"/>
       <x:c r="M2" s="9" t="str">
-        <x:v>是</x:v>
-      </x:c>
-      <x:c r="N2" s="9" t="str"/>
-      <x:c r="O2" s="9" t="str">
         <x:v>2026-06-10 20:15:32</x:v>
-      </x:c>
-      <x:c r="P2" s="9" t="str">
-        <x:v>待处理</x:v>
-      </x:c>
-      <x:c r="Q2" s="9" t="str">
-        <x:v>示例数据</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -373,38 +391,26 @@
         <x:v>黄丽</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>材料检查</x:v>
+        <x:v>新增成功</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
-        <x:v>导入成功</x:v>
+        <x:v>必传合同缺失</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>必传合同缺失</x:v>
-      </x:c>
-      <x:c r="I3" s="9" t="str">
         <x:v>文件信息-电子签章授权书</x:v>
       </x:c>
-      <x:c r="J3" s="9" t="str"/>
+      <x:c r="I3" s="9" t="str"/>
+      <x:c r="J3" s="9" t="str">
+        <x:v>电子签章授权书未上传，案件为未生效状态</x:v>
+      </x:c>
       <x:c r="K3" s="9" t="str">
-        <x:v>电子签章授权书未上传</x:v>
+        <x:v>否</x:v>
       </x:c>
       <x:c r="L3" s="9" t="str">
-        <x:v>进入材料补传页补齐必传合同</x:v>
+        <x:v>电子签章授权书</x:v>
       </x:c>
       <x:c r="M3" s="9" t="str">
-        <x:v>否</x:v>
-      </x:c>
-      <x:c r="N3" s="9" t="str">
-        <x:v>电子签章授权书</x:v>
-      </x:c>
-      <x:c r="O3" s="9" t="str">
         <x:v>2026-06-10 20:15:32</x:v>
-      </x:c>
-      <x:c r="P3" s="9" t="str">
-        <x:v>待补传</x:v>
-      </x:c>
-      <x:c r="Q3" s="9" t="str">
-        <x:v>示例数据</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -424,36 +430,24 @@
         <x:v>李明</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>订单关系检查</x:v>
+        <x:v>导入失败</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
-        <x:v>阻断失败</x:v>
+        <x:v>主续关系异常</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>主续关系异常</x:v>
-      </x:c>
-      <x:c r="I4" s="9" t="str">
         <x:v>订单基础信息-父订单编号</x:v>
       </x:c>
-      <x:c r="J4" s="9" t="str"/>
+      <x:c r="I4" s="9" t="str"/>
+      <x:c r="J4" s="9" t="str">
+        <x:v>续租订单未匹配到首租订单</x:v>
+      </x:c>
       <x:c r="K4" s="9" t="str">
-        <x:v>续租订单未匹配到首租订单</x:v>
-      </x:c>
-      <x:c r="L4" s="9" t="str">
-        <x:v>补充首租订单或确认系统内已存在首租订单</x:v>
-      </x:c>
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L4" s="9" t="str"/>
       <x:c r="M4" s="9" t="str">
-        <x:v>是</x:v>
-      </x:c>
-      <x:c r="N4" s="9" t="str"/>
-      <x:c r="O4" s="9" t="str">
         <x:v>2026-06-10 20:15:32</x:v>
-      </x:c>
-      <x:c r="P4" s="9" t="str">
-        <x:v>待处理</x:v>
-      </x:c>
-      <x:c r="Q4" s="9" t="str">
-        <x:v>示例数据</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>